<commit_message>
Cateos sin peticionante: rescatar casos con '/' y etiquetar 'sin peticionante publicado'
- parser: el titular 'se ha presentado X / ...' ahora corta bien en '/' y 'en el'.
- visor: cateos/servidumbres sin nombre muestran 'sin peticionante publicado'
  (el boletín no lo publica y la capa de permisos del catastro no trae titular).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out_hist/pedimentos.xlsx
+++ b/out_hist/pedimentos.xlsx
@@ -13464,6 +13464,11 @@
           <t>1124-585-G-22</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Golden Mining S.A</t>
+        </is>
+      </c>
       <c r="D270" t="inlineStr"/>
       <c r="E270" t="inlineStr">
         <is>
@@ -16382,6 +16387,11 @@
       <c r="A327" t="inlineStr">
         <is>
           <t>1124-573-G-25</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Glencore Pachon S.A</t>
         </is>
       </c>
       <c r="D327" t="inlineStr"/>

</xml_diff>

<commit_message>
Actualización completa: padrón WFS fresco + cruce + sociedades + histórico
Regenera toda la data derivada con el código actual y el padrón del WFS al día:
- descargar_padron (WFS): catastro/*.geojson.
- cruce boletín↔catastro: modelo.json (790/818 con match, incluye fechaInscripcionMensura).
- sociedades.json (418 entidades; ranking Cateos/Manifestaciones/Mensura en trámite/
  Mensura efectiva — Andes Corp. Minera #1 en efectiva con 19.664 ha).
- analisis_historico.json (áreas vacantes + antigüedad + zonas).
- pedimentos.geojson/xlsx regenerados desde el modelo. 818 expedientes intactos, 0 basura.
No se re-escaneó el boletín (sin cambios; el modelo ya tiene las mejoras del parser).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out_hist/pedimentos.xlsx
+++ b/out_hist/pedimentos.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>el pedido de mensura y caducar sus derechos</t>
+          <t>SCALZOTTO IDA FLORENCIA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -630,7 +630,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>I.P.E.E.M., so- licitando la Mensura de la mina “J XIV”</t>
+          <t>I.P.E.E.M</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -742,6 +742,11 @@
           <t>1124-438-K-17</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>KALIEROF, SERGIO DANIEL Y ASWELL S.A</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>oro</t>
@@ -853,6 +858,11 @@
           <t>156107-B-73</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KALIEROF, SERGIO DANIEL Y ASWELL S.A</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>oro</t>
@@ -1341,6 +1351,11 @@
           <t>1124.005-P-19</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ARGENTINA MINERA S.A</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>oro</t>
@@ -1441,6 +1456,11 @@
           <t>1124.015-P-19</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SEBASTIAN YAPUR MARZO</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
@@ -1603,6 +1623,11 @@
           <t>1124.086-A-19</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ARGENTINA MINERA S.A</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>oro</t>
@@ -1712,6 +1737,11 @@
           <t>1124.537A-18</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ARGENTINA MINERA S.A</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>oro</t>
@@ -2160,6 +2190,11 @@
           <t>1124-319-1-17</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>INSTITUTO PROVINCIAL DE EXPLORACIONES Y EXPLOTACIONES MINERAS LP.E.E.M</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>cobre</t>
@@ -2211,7 +2246,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DESARROLLO DE PROSPECTOS MINEROS S.A. Publíquese Edicto 2 veces</t>
+          <t>DESARROLLO DE PROSPECTOS MINEROS S.A</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -2419,7 +2454,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>BASTIAS GABRIEL ENRIQUE. Publíquese Edicto 2 veces</t>
+          <t>BASTIAS GABRIEL ENRIQUE</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2531,7 +2566,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BASTIAS GABRIEL ENRIQUE. Publíquese Edicto 2 veces</t>
+          <t>BASTIAS GABRIEL ENRIQUE</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2758,7 +2793,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BASTIAS YACANTE MARIA LAURA. Publíquese Edicto 2 veces</t>
+          <t>BASTIAS YACANTE MARIA LAURA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2861,6 +2896,11 @@
           <t>520-626-S-97</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>DESARROLLO DE RECURSOS S.A</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>oro</t>
@@ -3125,6 +3165,11 @@
           <t>1124-174-V-18</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>VILLAFAÑE MARIO ALBERTO</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
@@ -3220,6 +3265,11 @@
           <t>1124-241-P-2018</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PÁEZ RICARDO FRANCISCO</t>
+        </is>
+      </c>
       <c r="C53" t="inlineStr">
         <is>
           <t>Expte. 1124-545218-94</t>
@@ -3327,6 +3377,11 @@
           <t>1124-314-V-19</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>VERÓNICA LORENA VARGAS</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
@@ -3475,6 +3530,11 @@
           <t>1124-349-V-19</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>VERÓNICA LORENA VARGAS</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
@@ -3520,6 +3580,11 @@
           <t>1124-384-E-16</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>ECOMINING S.A</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
@@ -3618,6 +3683,11 @@
           <t>1124-401-G-2017</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>GRAMAGE ROLANDO NESTOR</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
@@ -3722,7 +3792,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ALCRUZ S.A. Publíquese Edicto 2 veces</t>
+          <t>ALCRUZ S.A</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3782,6 +3852,11 @@
           <t>1124-495-1-20</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>I.P.E.E.M</t>
+        </is>
+      </c>
       <c r="C64" t="inlineStr">
         <is>
           <t>Expte. 1124-545218-94</t>
@@ -3890,6 +3965,11 @@
           <t>545-748-H-94</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>MIRANDA S.A</t>
+        </is>
+      </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
@@ -4198,6 +4278,11 @@
           <t>1124-423-B-16</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ALCRUZ S.A</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
@@ -4379,7 +4464,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>?||expte. n9 1124-211-m-15. -</t>
+          <t>?|minas argentinas s.a|expte. n9 1124-211-m-15. -</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>MINAS ARGENTINAS S.A</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4496,6 +4586,11 @@
           <t>1124-183-Y-19</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>YAMANA ARGENTINAS SERVICIOS S.A</t>
+        </is>
+      </c>
       <c r="D78" t="inlineStr">
         <is>
           <t>oro</t>
@@ -4547,7 +4642,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>COLQUE EXPLORACIONES S.A. Publíquese Edicto 2 veces</t>
+          <t>COLQUE EXPLORACIONES S.A</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4602,7 +4697,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>la Empresa Desarrollo de Recursos S.A</t>
+          <t>Desarrollo de Recursos S.A</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4855,7 +4950,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>BASTIAS HUGO ENRIQUE. Publíquese Edicto 2 veces</t>
+          <t>BASTIAS HUGO ENRIQUE</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
@@ -4908,7 +5003,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>la Empresa Argentina Minera S.A</t>
+          <t>Argentina Minera S.A</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -5075,7 +5170,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>GABRIEL ENRIQUE BASTIAS. Publíquese Edicto 2 veces</t>
+          <t>GABRIEL ENRIQUE BASTIAS</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
@@ -5125,7 +5220,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>GABRIEL ENRIQUE BASTIAS. Publíquese Edicto 2 veces</t>
+          <t>GABRIEL ENRIQUE BASTIAS</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
@@ -5234,7 +5329,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>AURORA MINING S.A. Publíquese Edicto 2 veces</t>
+          <t>AURORA MINING S.A</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
@@ -5343,7 +5438,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>GABRIEL ENRIQUE BASTIAS. Publíquese Edicto 2 veces</t>
+          <t>GABRIEL ENRIQUE BASTIAS</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
@@ -5623,7 +5718,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>BASTIAS HUGO ENRIQUE. Publíquese Edicto 2 veces</t>
+          <t>BASTIAS HUGO ENRIQUE</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5675,6 +5770,11 @@
           <t>1124-017-B-21</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>BASTIAS GABRIEL ENRIQUE</t>
+        </is>
+      </c>
       <c r="D100" t="inlineStr">
         <is>
           <t>oro</t>
@@ -5887,6 +5987,11 @@
           <t>1124-385-C-19</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>CARRIZO ANGEL IGNACIO Y ONTIVERO ARIEL MARIO</t>
+        </is>
+      </c>
       <c r="D104" t="inlineStr">
         <is>
           <t>cuarzo</t>
@@ -6285,7 +6390,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Gramage GABRIEL ENRIQUE BASTIAS. Publíquese Edicto 2 veces</t>
+          <t>Gramage GABRIEL ENRIQUE BASTIAS</t>
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
@@ -6335,7 +6440,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>BASTIAS YACANTE GABRIEL ENRIQUE. Publíquese Edicto 2 veces</t>
+          <t>BASTIAS YACANTE GABRIEL ENRIQUE</t>
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
@@ -6388,7 +6493,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Gramage GABRIEL ENRIQUE BASTIAS. Publíquese Edicto 2 veces</t>
+          <t>Gramage GABRIEL ENRIQUE BASTIAS</t>
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
@@ -6438,7 +6543,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>CEBALLOS MAIZ JUAN PABLO Y LARA ROBERTO. Publíquese Edicto 2</t>
+          <t>CEBALLOS MAIZ JUAN PABLO Y LARA ROBERTO</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
@@ -6488,7 +6593,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>COLQUE EXPLORACIONES S.A. Publíquese Edicto 2 veces</t>
+          <t>COLQUE EXPLORACIONES S.A</t>
         </is>
       </c>
       <c r="D117" t="inlineStr"/>
@@ -6597,7 +6702,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>MIRANDA S.A. Publíquese Edicto 2 veces</t>
+          <t>MIRANDA S.A</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -6654,7 +6759,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Gramage MARIA LAURA BASTIAS YACANTE. Publíquese Edicto 2 veces</t>
+          <t>Gramage MARIA LAURA BASTIAS YACANTE</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -6889,6 +6994,11 @@
           <t>296.775-G-90</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>MINERA DEL CARMEN S.A</t>
+        </is>
+      </c>
       <c r="D124" t="inlineStr">
         <is>
           <t>oro</t>
@@ -7059,7 +7169,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>HUGO ENRIQUE BASTIAS. Publíquese Edicto 2 veces</t>
+          <t>HUGO ENRIQUE BASTIAS</t>
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
@@ -7109,7 +7219,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>RAUL ERNESTO CONCINA. Publíquese Edicto 2 veces</t>
+          <t>RAUL ERNESTO CONCINA</t>
         </is>
       </c>
       <c r="D128" t="inlineStr"/>
@@ -7218,7 +7328,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>DESARROLLO DE RECURSOS S.A. Publíquese Edicto 2 veces</t>
+          <t>DESARROLLO DE RECURSOS S.A</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -7273,6 +7383,11 @@
           <t>1124-225-T-13</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>CASPOSO ARGENTINA LTD. SUCURSAL</t>
+        </is>
+      </c>
       <c r="D131" t="inlineStr">
         <is>
           <t>oro</t>
@@ -7324,7 +7439,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>BASTIAS YACANTE MARIA LAURA. Sucursal. Publíquese Edicto 2 veces</t>
+          <t>BASTIAS YACANTE MARIA LAURA. Sucursal</t>
         </is>
       </c>
       <c r="D132" t="inlineStr"/>
@@ -7372,6 +7487,11 @@
           <t>1124-323-1-17</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>I.P.E.E.M</t>
+        </is>
+      </c>
       <c r="D133" t="inlineStr">
         <is>
           <t>oro</t>
@@ -7646,6 +7766,11 @@
           <t>1207-B-96</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>BARRICK EXPLORACIONES ARGENTINA S.A</t>
+        </is>
+      </c>
       <c r="D138" t="inlineStr">
         <is>
           <t>oro</t>
@@ -7813,7 +7938,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>PETRA GOLD SERVICIOS MINEROS S.R.L. Publíquese Edicto 2 veces</t>
+          <t>PETRA GOLD SERVICIOS MINEROS S.R.L</t>
         </is>
       </c>
       <c r="D141" t="inlineStr"/>
@@ -7928,7 +8053,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>CASPOSO ARGENTINA LTD. SUCURSAL. Publíquese Edicto 2 veces</t>
+          <t>CASPOSO ARGENTINA LTD. SUCURSAL</t>
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
@@ -7981,7 +8106,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>CASPOSO ARGENTINA LTD. SUCURSAL ARGENTINA. Publíquese Edicto</t>
+          <t>CASPOSO ARGENTINA LTD. SUCURSAL ARGENTINA</t>
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
@@ -8032,6 +8157,11 @@
           <t>425-294-M-02</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>YAMANA ARGENTINA SERVICIOS S.A</t>
+        </is>
+      </c>
       <c r="D145" t="inlineStr">
         <is>
           <t>oro</t>
@@ -8086,7 +8216,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>MIRANDA S.A. Publíquese Edicto 2 veces</t>
+          <t>MIRANDA S.A</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
@@ -8258,6 +8388,11 @@
           <t>1124-016-B-20</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>BASTIAS HUGO ENRIQUE</t>
+        </is>
+      </c>
       <c r="D149" t="inlineStr">
         <is>
           <t>oro</t>
@@ -8368,7 +8503,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>CORDON DEL NORTE S.A. Publíquese Edicto 2 veces</t>
+          <t>CORDON DEL NORTE S.A</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
@@ -8532,6 +8667,11 @@
           <t>1124-250-B-20</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>BASTIAS YACANTE GABRIEL ENRIQUE</t>
+        </is>
+      </c>
       <c r="D154" t="inlineStr">
         <is>
           <t>oro</t>
@@ -8584,6 +8724,11 @@
           <t>1124-256-D-20</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>I.P.E.E.M</t>
+        </is>
+      </c>
       <c r="D155" t="inlineStr">
         <is>
           <t>oro</t>
@@ -8633,6 +8778,11 @@
           <t>1124-290-A-21</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>AURORA MINING S.A</t>
+        </is>
+      </c>
       <c r="D156" t="inlineStr">
         <is>
           <t>oro</t>
@@ -8743,7 +8893,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>DEPROMINSA. Publíquese Edicto 2 veces</t>
+          <t>DEPROMINSA</t>
         </is>
       </c>
       <c r="D158" t="inlineStr"/>
@@ -8793,7 +8943,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>MINERA SUD ARGENTINA S.A. Publíquese Edicto 2 veces</t>
+          <t>MINERA SUD ARGENTINA S.A</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -8850,7 +9000,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CORDON DEL NORTE S.A. Publíquese Edicto 2 veces</t>
+          <t>CORDON DEL NORTE S.A</t>
         </is>
       </c>
       <c r="D160" t="inlineStr"/>
@@ -8957,7 +9107,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>DESARROLLO DE RECURSOS S.A. Publíquese Edicto 2 veces</t>
+          <t>DESARROLLO DE RECURSOS S.A</t>
         </is>
       </c>
       <c r="D162" t="inlineStr"/>
@@ -9060,7 +9210,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>HUGO ENRIQUE BASTIAS. Publíquese Edicto 2 veces</t>
+          <t>HUGO ENRIQUE BASTIAS</t>
         </is>
       </c>
       <c r="D164" t="inlineStr"/>
@@ -9110,7 +9260,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>GABRIEL ENRIQUE BASTIAS. Publíquese Edicto 2 veces</t>
+          <t>GABRIEL ENRIQUE BASTIAS</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -9162,6 +9312,11 @@
           <t>1124-61-C-11</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>COLQUE EXPLORACIONES S.A</t>
+        </is>
+      </c>
       <c r="D166" t="inlineStr">
         <is>
           <t>oro</t>
@@ -9396,7 +9551,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CASPOSO ARGENTINA LTD. Sucursal. Publíquese Edicto 2 veces</t>
+          <t>CASPOSO ARGENTINA LTD. Sucursal</t>
         </is>
       </c>
       <c r="D170" t="inlineStr"/>
@@ -9503,7 +9658,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>MIRANDA S.A. Publíquese Edicto 2 veces</t>
+          <t>MIRANDA S.A</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -9675,7 +9830,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>por acciones escriturales de $</t>
+          <t>BASTIAS LUIS ABELARDO (SUC).” e</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -9786,6 +9941,11 @@
           <t>242.984-M-87</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>MINERA DEL CARMEN S.A</t>
+        </is>
+      </c>
       <c r="D177" t="inlineStr">
         <is>
           <t>oro</t>
@@ -9837,7 +9997,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>el |.P.E.E.M</t>
+          <t>|.P.E.E.M</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -9896,7 +10056,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>MIRANDA S.A. Publíquese Edicto 2 veces</t>
+          <t>MIRANDA S.A</t>
         </is>
       </c>
       <c r="D179" t="inlineStr"/>
@@ -9947,6 +10107,11 @@
           <t>558-L-95</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>MIRANDA S.A</t>
+        </is>
+      </c>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
@@ -9989,12 +10154,12 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>?iglesia|el i.p.e.e.m|de autos. se tienen presentes</t>
+          <t>?iglesia|i.p.e.e.m|de autos. se tienen presentes</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>el I.P.E.E.M</t>
+          <t>I.P.E.E.M</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -10053,7 +10218,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>SUAREZ HUGO GERONIMO. Publíquese Edicto 2 veces</t>
+          <t>SUAREZ HUGO GERONIMO</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -10267,6 +10432,11 @@
           <t>1124-298-B-21</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>HUGO A. BOSQUE Y DINA MYRIAM ELIZONDO</t>
+        </is>
+      </c>
       <c r="D186" t="inlineStr">
         <is>
           <t>oro</t>
@@ -10316,6 +10486,11 @@
           <t>1124-421-B-20</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>HUGO A. BOSQUE</t>
+        </is>
+      </c>
       <c r="C187" t="inlineStr">
         <is>
           <t>U.T</t>
@@ -10480,7 +10655,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Gramage ROLANDO NESTOR. Publíquese Edicto 2 veces</t>
+          <t>Gramage ROLANDO NESTOR</t>
         </is>
       </c>
       <c r="D190" t="inlineStr"/>
@@ -10873,7 +11048,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Dionisio Ramos</t>
+          <t>FUENTES VICTOR GUILLERMO Y FUENTES VICTOR HERIBERTO</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -11472,6 +11647,11 @@
           <t>1124-305-B-21</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>BOSQUE HUGO ARTURO Y MANINI GARCIA MARTHA CAROLINA</t>
+        </is>
+      </c>
       <c r="D208" t="inlineStr">
         <is>
           <t>plata</t>
@@ -11629,6 +11809,11 @@
           <t>1124-386-M-13</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>BOSQUE HUGO ARTURO</t>
+        </is>
+      </c>
       <c r="D211" t="inlineStr">
         <is>
           <t>oro</t>
@@ -11678,6 +11863,11 @@
           <t>1124-437-A-20</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>ARGENTINA MINERA S.A</t>
+        </is>
+      </c>
       <c r="D212" t="inlineStr">
         <is>
           <t>oro</t>
@@ -11732,7 +11922,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>“MINERA SUD ARGENTINA S.A.”</t>
+          <t>BOSQUE HUGO ARTURO</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -11787,6 +11977,11 @@
           <t>1124-531-B-18</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>BOSQUE HUGO ARTURO</t>
+        </is>
+      </c>
       <c r="D214" t="inlineStr">
         <is>
           <t>oro</t>
@@ -11836,6 +12031,11 @@
           <t>1124-561-L-19</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>LOVERA JUAN JOSE Y LOVERA JUAN ANGEL</t>
+        </is>
+      </c>
       <c r="C215" t="inlineStr">
         <is>
           <t>EXPTE</t>
@@ -12322,6 +12522,11 @@
           <t>545.927-L-94</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>PETRA GOLD SERVICIOS MINEROS S.R.L</t>
+        </is>
+      </c>
       <c r="D224" t="inlineStr">
         <is>
           <t>oro</t>
@@ -12374,6 +12579,11 @@
           <t>1124-000334-1-2021</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>I.P.E.E.M</t>
+        </is>
+      </c>
       <c r="D225" t="inlineStr">
         <is>
           <t>oro</t>
@@ -12634,6 +12844,11 @@
           <t>1124-449-M-21</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>MIRANDA S.A</t>
+        </is>
+      </c>
       <c r="D230" t="inlineStr">
         <is>
           <t>oro</t>
@@ -13366,6 +13581,11 @@
           <t>1124-344-S-10</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>HUGO ARTURO BOSQUE</t>
+        </is>
+      </c>
       <c r="D244" t="inlineStr">
         <is>
           <t>oro</t>
@@ -13629,6 +13849,11 @@
           <t>1124-530-B-2012</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>HUGO ARTURO BOSQUE</t>
+        </is>
+      </c>
       <c r="D249" t="inlineStr">
         <is>
           <t>cobre, oro</t>
@@ -14665,6 +14890,11 @@
           <t>1124-253-8-21</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>FUENTES VICTOR GUILLERMO Y FUENTES VICTOR HERIBERTO</t>
+        </is>
+      </c>
       <c r="D268" t="inlineStr">
         <is>
           <t>oro</t>
@@ -15082,6 +15312,11 @@
           <t>1124-338-M-21</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>MAIDANA JULIAN SANTIAGO</t>
+        </is>
+      </c>
       <c r="D276" t="inlineStr"/>
       <c r="E276" t="inlineStr">
         <is>
@@ -15347,6 +15582,11 @@
           <t>1124-409-S-21</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>FUENTES VICTOR GUILLERMO</t>
+        </is>
+      </c>
       <c r="C281" t="inlineStr">
         <is>
           <t>Expte. 119-B-50</t>
@@ -15401,6 +15641,11 @@
           <t>1124-422-B-20</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>BOSQUE HUGO ARTURO</t>
+        </is>
+      </c>
       <c r="D282" t="inlineStr">
         <is>
           <t>oro</t>
@@ -16196,6 +16441,11 @@
           <t>1124-035-D-22</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>DESARROLLO DE PROSPECTOS MINEROS S.A</t>
+        </is>
+      </c>
       <c r="D297" t="inlineStr">
         <is>
           <t>oro</t>
@@ -16358,6 +16608,11 @@
           <t>1124-282-S-06</t>
         </is>
       </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>BOSQUE HUGO ARTURO</t>
+        </is>
+      </c>
       <c r="D300" t="inlineStr">
         <is>
           <t>oro</t>
@@ -17113,6 +17368,11 @@
           <t>1124-198-S-14</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>SANCHEZ ARMANDO JESUS</t>
+        </is>
+      </c>
       <c r="D314" t="inlineStr">
         <is>
           <t>oro</t>
@@ -17207,6 +17467,11 @@
           <t>1124-252-S-21</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>VICTOR GUILLERMO FUENTES Y FUENTES VICTOR HERIBERTO</t>
+        </is>
+      </c>
       <c r="C316" t="inlineStr">
         <is>
           <t>Expte. 22-N-38</t>
@@ -17500,7 +17765,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>“COMPAÑÍA MINERA PIUQUENES S.A.”.- Publíquese</t>
+          <t>“COMPAÑÍA MINERA PIUQUENES S.A.”</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
@@ -17552,6 +17817,11 @@
           <t>414850-S-05</t>
         </is>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>SANCHEZ ARMANDO JESUS</t>
+        </is>
+      </c>
       <c r="C323" t="inlineStr">
         <is>
           <t>Expte. 22-N-38</t>
@@ -17609,6 +17879,11 @@
           <t>461-B-95</t>
         </is>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>HUGO ENRIQUE BASTIAS</t>
+        </is>
+      </c>
       <c r="D324" t="inlineStr">
         <is>
           <t>oro</t>
@@ -18094,6 +18369,11 @@
           <t>1124-404-P-21</t>
         </is>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>GASTON PELUC MAURIN Y ALEJANDRO PELUC MAURIN</t>
+        </is>
+      </c>
       <c r="D333" t="inlineStr">
         <is>
           <t>cuarzo</t>
@@ -18576,6 +18856,11 @@
           <t>296.783-N-90</t>
         </is>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>MINERA DEL CARMEN S.A</t>
+        </is>
+      </c>
       <c r="D342" t="inlineStr">
         <is>
           <t>oro</t>
@@ -19971,6 +20256,11 @@
           <t>1124-567-A-19</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>ARGENTINA MINERA 5S.A</t>
+        </is>
+      </c>
       <c r="D368" t="inlineStr">
         <is>
           <t>oro</t>
@@ -20727,6 +21017,11 @@
           <t>1124-448-M-21</t>
         </is>
       </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>MIRANDA S.A</t>
+        </is>
+      </c>
       <c r="D382" t="inlineStr">
         <is>
           <t>oro</t>
@@ -21206,6 +21501,11 @@
           <t>545.605-C-94</t>
         </is>
       </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>GOLDEN MINING S.A. Y ALIAS RICARDO ROMERO</t>
+        </is>
+      </c>
       <c r="D391" t="inlineStr">
         <is>
           <t>cobre</t>
@@ -22530,7 +22830,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>“GOLDEN</t>
+          <t>AGUILERA MARIO RAUL</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
@@ -22639,6 +22939,11 @@
           <t>1124-157-1-23</t>
         </is>
       </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>L.P.E.E.M</t>
+        </is>
+      </c>
       <c r="D419" t="inlineStr">
         <is>
           <t>plata</t>
@@ -22733,6 +23038,11 @@
           <t>1124-203-1-22</t>
         </is>
       </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>LP.E.E.M</t>
+        </is>
+      </c>
       <c r="D421" t="inlineStr">
         <is>
           <t>plata</t>
@@ -22782,6 +23092,11 @@
           <t>1124-206-B-22</t>
         </is>
       </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>BASTIAS GABRIEL ENRIQUE</t>
+        </is>
+      </c>
       <c r="C422" t="inlineStr">
         <is>
           <t>EXPTE</t>
@@ -23027,6 +23342,11 @@
           <t>1124-420-S-22</t>
         </is>
       </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>SABLE ARGENTINA S.A</t>
+        </is>
+      </c>
       <c r="C427" t="inlineStr">
         <is>
           <t>EXPTE</t>
@@ -23292,6 +23612,11 @@
           <t>1124-528-L-21</t>
         </is>
       </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>BASTIAS GABRIEL ENRIQUE</t>
+        </is>
+      </c>
       <c r="D432" t="inlineStr">
         <is>
           <t>oro</t>
@@ -23488,6 +23813,11 @@
           <t>1124-108-G-22</t>
         </is>
       </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>GOLDEN MINING S.A</t>
+        </is>
+      </c>
       <c r="C436" t="inlineStr">
         <is>
           <t>Expte. 258852-P-84</t>
@@ -23584,6 +23914,11 @@
           <t>1124-404-B-22</t>
         </is>
       </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Clemente Chirapozo lo que se</t>
+        </is>
+      </c>
       <c r="C438" t="inlineStr">
         <is>
           <t>Expte. 373-P-48</t>
@@ -23641,6 +23976,11 @@
           <t>1124-424-0-22</t>
         </is>
       </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>OLIVARES S.A</t>
+        </is>
+      </c>
       <c r="C439" t="inlineStr">
         <is>
           <t>Expte. 258852-P-84</t>
@@ -24639,6 +24979,11 @@
           <t>1124-325-C-22</t>
         </is>
       </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>CASPOSO ARGENTINA LTD</t>
+        </is>
+      </c>
       <c r="D459" t="inlineStr">
         <is>
           <t>oro</t>
@@ -24826,6 +25171,11 @@
           <t>1124-464-M-09</t>
         </is>
       </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Denel S.A. No esta vigente, por haber sido</t>
+        </is>
+      </c>
       <c r="D463" t="inlineStr"/>
       <c r="E463" t="inlineStr">
         <is>
@@ -25350,6 +25700,11 @@
           <t>1124-048-M-22</t>
         </is>
       </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Productos Frescos S.A. (No Costa CUIT), las</t>
+        </is>
+      </c>
       <c r="D474" t="inlineStr"/>
       <c r="E474" t="inlineStr">
         <is>
@@ -25395,6 +25750,11 @@
           <t>1124-052-1-22</t>
         </is>
       </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>I.P.E.E.M</t>
+        </is>
+      </c>
       <c r="C475" t="inlineStr">
         <is>
           <t>EXPTE</t>
@@ -25449,6 +25809,11 @@
           <t>1124-073-M-22</t>
         </is>
       </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>GWK MINERALS S$.A</t>
+        </is>
+      </c>
       <c r="D476" t="inlineStr">
         <is>
           <t>oro</t>
@@ -25785,6 +26150,11 @@
           <t>1124-564-G-21</t>
         </is>
       </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Plana salas Mario Luis D.N.I.N* 10</t>
+        </is>
+      </c>
       <c r="D483" t="inlineStr"/>
       <c r="E483" t="inlineStr">
         <is>
@@ -25975,6 +26345,11 @@
           <t>545.864-G-94</t>
         </is>
       </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>GWK MINERALS S.A</t>
+        </is>
+      </c>
       <c r="D487" t="inlineStr">
         <is>
           <t>oro</t>
@@ -26083,6 +26458,11 @@
           <t>1124-364-1-2020</t>
         </is>
       </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>I.P.E.E.M</t>
+        </is>
+      </c>
       <c r="D489" t="inlineStr">
         <is>
           <t>oro</t>
@@ -26366,6 +26746,11 @@
           <t>1124-549-A-22</t>
         </is>
       </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Martinez Rogelio</t>
+        </is>
+      </c>
       <c r="D495" t="inlineStr">
         <is>
           <t>oro</t>
@@ -27885,6 +28270,11 @@
           <t>1124</t>
         </is>
       </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>BAMASA MINING SERVICES S.R.L</t>
+        </is>
+      </c>
       <c r="D525" t="inlineStr">
         <is>
           <t>oro</t>
@@ -28161,7 +28551,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>"BAMASA MINING SERVICES S.R.L.”, publíquese Edicto 2 veces</t>
+          <t>"BAMASA MINING SERVICES S.R.L.”</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
@@ -28218,7 +28608,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>la empresa PACHON S.A</t>
+          <t>PACHON S.A</t>
         </is>
       </c>
       <c r="D532" t="inlineStr"/>
@@ -28555,6 +28945,11 @@
           <t>1124-204-1-2022</t>
         </is>
       </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>ILP.E.E.M</t>
+        </is>
+      </c>
       <c r="C539" t="inlineStr">
         <is>
           <t>EXPTE. NS 1124-204-1-2022</t>
@@ -28609,6 +29004,11 @@
           <t>1124-239-M-23</t>
         </is>
       </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>I.P.E.E.M</t>
+        </is>
+      </c>
       <c r="D540" t="inlineStr">
         <is>
           <t>oro, plata</t>
@@ -29044,6 +29444,11 @@
           <t>1124-53</t>
         </is>
       </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>NUEVA GRAN VICTORIA S.A</t>
+        </is>
+      </c>
       <c r="D549" t="inlineStr">
         <is>
           <t>cobre</t>
@@ -29182,6 +29587,11 @@
           <t>1124-5953</t>
         </is>
       </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>NUEVA GRAN VICTORIA S$.A</t>
+        </is>
+      </c>
       <c r="D552" t="inlineStr">
         <is>
           <t>cobre</t>
@@ -29231,6 +29641,11 @@
           <t>1124-666-B-2022</t>
         </is>
       </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>HUGO ARTURO BOSQUE</t>
+        </is>
+      </c>
       <c r="D553" t="inlineStr">
         <is>
           <t>oro</t>
@@ -29382,6 +29797,11 @@
           <t>1124-067-B-23</t>
         </is>
       </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>SABLE ARGENTINA S.A</t>
+        </is>
+      </c>
       <c r="C557" t="inlineStr">
         <is>
           <t>Expte. 3621-G-64</t>
@@ -29480,6 +29900,11 @@
           <t>1124-142-B-23</t>
         </is>
       </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>SABLE ARGENTINA S.A</t>
+        </is>
+      </c>
       <c r="C559" t="inlineStr">
         <is>
           <t>Expte. 2212-M-58</t>
@@ -29624,6 +30049,11 @@
           <t>1124-243-M-21</t>
         </is>
       </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>BASTIAS YACANTE MARIA LAURA</t>
+        </is>
+      </c>
       <c r="D562" t="inlineStr">
         <is>
           <t>oro</t>
@@ -29810,6 +30240,11 @@
           <t>1124-428-0-2022</t>
         </is>
       </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>SABLE ARGENTINA S.A</t>
+        </is>
+      </c>
       <c r="C566" t="inlineStr">
         <is>
           <t>Expte. 3621-G-64</t>
@@ -29864,6 +30299,11 @@
           <t>1124-446-D-2022</t>
         </is>
       </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>COLIN GEOFFREY</t>
+        </is>
+      </c>
       <c r="D567" t="inlineStr">
         <is>
           <t>oro</t>
@@ -29958,6 +30398,11 @@
           <t>1124-593</t>
         </is>
       </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>NUEVA GRAN VICTORIA $.A</t>
+        </is>
+      </c>
       <c r="D569" t="inlineStr">
         <is>
           <t>cobre</t>
@@ -30046,6 +30491,11 @@
           <t>1124-595-L-22</t>
         </is>
       </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Leyes Braulio</t>
+        </is>
+      </c>
       <c r="D571" t="inlineStr"/>
       <c r="E571" t="inlineStr">
         <is>
@@ -30847,6 +31297,11 @@
           <t>1124-126-N-2022</t>
         </is>
       </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>NUEVA GRAN VICTORIA S.A</t>
+        </is>
+      </c>
       <c r="D589" t="inlineStr">
         <is>
           <t>cobre</t>
@@ -30896,6 +31351,11 @@
           <t>1124-127-N-2022</t>
         </is>
       </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>NUEVA GRAN VICTORIA S.A</t>
+        </is>
+      </c>
       <c r="D590" t="inlineStr">
         <is>
           <t>cobre</t>
@@ -31154,6 +31614,11 @@
           <t>1124-484-B-2023</t>
         </is>
       </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>BAMASA MINING SERVICES S.R.L</t>
+        </is>
+      </c>
       <c r="C595" t="inlineStr">
         <is>
           <t>EXPTE</t>
@@ -31503,6 +31968,11 @@
           <t>1124-264-A-23</t>
         </is>
       </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Leyes Braulio</t>
+        </is>
+      </c>
       <c r="D602" t="inlineStr">
         <is>
           <t>oro</t>
@@ -31546,6 +32016,11 @@
           <t>1124-483-G-2022</t>
         </is>
       </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>GUARDIOLA GARCIA ARTURO</t>
+        </is>
+      </c>
       <c r="D603" t="inlineStr">
         <is>
           <t>oro</t>
@@ -31900,6 +32375,11 @@
           <t>1124-331-C-08</t>
         </is>
       </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>HUGO ENRIQUE BASTIAS</t>
+        </is>
+      </c>
       <c r="D610" t="inlineStr">
         <is>
           <t>caliza, oro</t>
@@ -31988,6 +32468,11 @@
           <t>1124-367-M-23</t>
         </is>
       </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>HUGO ENRIQUE BASTIAS</t>
+        </is>
+      </c>
       <c r="D612" t="inlineStr">
         <is>
           <t>oro</t>
@@ -32243,6 +32728,11 @@
           <t>302-F-199</t>
         </is>
       </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>HUGO ENRIQUE BASTIAS</t>
+        </is>
+      </c>
       <c r="D617" t="inlineStr">
         <is>
           <t>oro</t>
@@ -32611,6 +33101,11 @@
           <t>1124-401-B-23</t>
         </is>
       </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>PROYECTO HUACHI S.R.L</t>
+        </is>
+      </c>
       <c r="D625" t="inlineStr">
         <is>
           <t>oro</t>
@@ -32660,6 +33155,11 @@
           <t>1124-405-B-23</t>
         </is>
       </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Leyes Braulio</t>
+        </is>
+      </c>
       <c r="D626" t="inlineStr">
         <is>
           <t>oro</t>
@@ -32712,6 +33212,11 @@
           <t>1124-493-P-2020</t>
         </is>
       </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>PROYECTO HUACHI S.R.L</t>
+        </is>
+      </c>
       <c r="D627" t="inlineStr">
         <is>
           <t>oro</t>
@@ -33480,6 +33985,11 @@
           <t>1124-043-B-2024</t>
         </is>
       </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>BASTIAS YACANTE GABRIEL ENRIQUE</t>
+        </is>
+      </c>
       <c r="D644" t="inlineStr">
         <is>
           <t>oro, plata</t>
@@ -33531,7 +34041,7 @@
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>“OLIVARES S.A.- Publíquese</t>
+          <t>“OLIVARES S.A</t>
         </is>
       </c>
       <c r="D645" t="inlineStr">
@@ -33669,7 +34179,7 @@
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>“OLIVARES S.A.- Publíquese</t>
+          <t>“OLIVARES S.A</t>
         </is>
       </c>
       <c r="D648" t="inlineStr">
@@ -33866,6 +34376,11 @@
           <t>1124-356-T-24</t>
         </is>
       </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Fernández Maria Antonia L.C.N* 1</t>
+        </is>
+      </c>
       <c r="D652" t="inlineStr"/>
       <c r="E652" t="inlineStr">
         <is>
@@ -34546,6 +35061,11 @@
           <t>1124-072-B-2024</t>
         </is>
       </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>BAMASA MINING SERVICES S.A</t>
+        </is>
+      </c>
       <c r="D667" t="inlineStr">
         <is>
           <t>oro</t>
@@ -34784,6 +35304,11 @@
           <t>1124-225-T-2024</t>
         </is>
       </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Leonardi Aníbal Guillermo</t>
+        </is>
+      </c>
       <c r="D672" t="inlineStr"/>
       <c r="E672" t="inlineStr">
         <is>
@@ -34829,6 +35354,11 @@
           <t>1124-226-T-2024</t>
         </is>
       </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Leonardi Aníbal Guillermo</t>
+        </is>
+      </c>
       <c r="D673" t="inlineStr"/>
       <c r="E673" t="inlineStr">
         <is>
@@ -34913,6 +35443,11 @@
           <t>1124-243-B-24</t>
         </is>
       </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>AURORA MINING $.A</t>
+        </is>
+      </c>
       <c r="D675" t="inlineStr">
         <is>
           <t>oro</t>
@@ -35966,7 +36501,7 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>la empresa GWK MINERALS S.A</t>
+          <t>GWK MINERALS S.A</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
@@ -36064,6 +36599,11 @@
           <t>1124-399-A-2024</t>
         </is>
       </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>JAMAL S.A.S</t>
+        </is>
+      </c>
       <c r="D699" t="inlineStr">
         <is>
           <t>oro</t>
@@ -36630,6 +37170,11 @@
           <t>1124-642-A-2023</t>
         </is>
       </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>AURORA MINING S$.A</t>
+        </is>
+      </c>
       <c r="D711" t="inlineStr">
         <is>
           <t>oro</t>
@@ -36833,6 +37378,11 @@
           <t>546.314-A-94</t>
         </is>
       </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>AURORA MINING S.A</t>
+        </is>
+      </c>
       <c r="D715" t="inlineStr">
         <is>
           <t>oro</t>
@@ -36882,12 +37432,12 @@
     <row r="716">
       <c r="A716" t="inlineStr">
         <is>
-          <t>?iglesia|la empresa gwk minerals s.a|de autos. se tienen presentes</t>
+          <t>?iglesia|gwk minerals s.a|de autos. se tienen presentes</t>
         </is>
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>la empresa GWK MINERALS S.A</t>
+          <t>GWK MINERALS S.A</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
@@ -37399,6 +37949,11 @@
           <t>1124-051-L-2022</t>
         </is>
       </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>LOVERA JUAN JOSE, LOVERA JUAN ÁNGEL Y GABRIEL LUIS LAS HERAS</t>
+        </is>
+      </c>
       <c r="D726" t="inlineStr">
         <is>
           <t>oro</t>
@@ -37498,6 +38053,11 @@
           <t>1124-243-V-25</t>
         </is>
       </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>LOVERA JUAN JOSE, LOVERA JUAN ÁNGEL Y GABRIEL LUIS LAS HERAS</t>
+        </is>
+      </c>
       <c r="D728" t="inlineStr">
         <is>
           <t>oro</t>
@@ -38448,6 +39008,11 @@
           <t>1124-216-E-2023</t>
         </is>
       </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>ENTROPY RESOURCES S.A</t>
+        </is>
+      </c>
       <c r="D746" t="inlineStr">
         <is>
           <t>oro</t>
@@ -38856,6 +39421,11 @@
           <t>1124-660-B-2022</t>
         </is>
       </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>BOSQUE HUGO ARTURO</t>
+        </is>
+      </c>
       <c r="D754" t="inlineStr">
         <is>
           <t>hierro</t>
@@ -39293,6 +39863,11 @@
           <t>1124-411-C-2025</t>
         </is>
       </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>CALINGASTA MINERALES S.R.L</t>
+        </is>
+      </c>
       <c r="D763" t="inlineStr">
         <is>
           <t>bentonita</t>
@@ -39397,6 +39972,11 @@
           <t>1124-579-C-24</t>
         </is>
       </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>CALINGASTA MINERALES S.R.L</t>
+        </is>
+      </c>
       <c r="D765" t="inlineStr">
         <is>
           <t>bentonita</t>
@@ -39446,6 +40026,11 @@
           <t>1124-580-C-24</t>
         </is>
       </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>CALINGASTA MINERALES S.R.L</t>
+        </is>
+      </c>
       <c r="D766" t="inlineStr">
         <is>
           <t>bentonita</t>
@@ -39692,6 +40277,11 @@
           <t>1124-085-B-2024</t>
         </is>
       </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>BAMASA MINING SERVICES $S.R.L</t>
+        </is>
+      </c>
       <c r="D771" t="inlineStr">
         <is>
           <t>oro</t>
@@ -40794,6 +41384,11 @@
           <t>1124-258-X-2013</t>
         </is>
       </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>GLENCORE PACHON $.A</t>
+        </is>
+      </c>
       <c r="D792" t="inlineStr">
         <is>
           <t>plata</t>
@@ -41634,6 +42229,11 @@
           <t>1124-405-P-2017</t>
         </is>
       </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>PUENTE CLAUDIO</t>
+        </is>
+      </c>
       <c r="D808" t="inlineStr">
         <is>
           <t>bentonita</t>
@@ -41735,7 +42335,7 @@
       </c>
       <c r="B810" t="inlineStr">
         <is>
-          <t>Minera del Carmen S.A</t>
+          <t>BOSQUE HUGO ARTURO</t>
         </is>
       </c>
       <c r="D810" t="inlineStr">

</xml_diff>